<commit_message>
Rename Ramesh Dinge to Ramesh Ginde and regenerate signatures
</commit_message>
<xml_diff>
--- a/employees/employees.xlsx
+++ b/employees/employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Email Signature\employees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058CCB02-D191-4B52-ACEE-AED1F137C34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF9C713F-B206-404C-90CC-AA2B94D51563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{13FF4E98-4AD7-478F-BA3A-EC3DF8F57A6B}"/>
   </bookViews>
@@ -80,9 +80,6 @@
     <t>mayuri@abhinavgroup.co.in</t>
   </si>
   <si>
-    <t>Ramesh Dinge</t>
-  </si>
-  <si>
     <t>Architect</t>
   </si>
   <si>
@@ -132,6 +129,9 @@
   </si>
   <si>
     <t>xyz@gmail.com</t>
+  </si>
+  <si>
+    <t>Ramesh Ginde</t>
   </si>
 </sst>
 </file>
@@ -598,86 +598,86 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>18</v>
       </c>
       <c r="C6" s="2">
         <v>9309505388</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
       </c>
       <c r="C7">
         <v>7219550051</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>24</v>
       </c>
       <c r="C8">
         <v>7219550010</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
       </c>
       <c r="C9">
         <v>9588623420</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
         <v>29</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
       </c>
       <c r="C10">
         <v>1234567890</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate 4 new employee signatures: Anjan, Hemant, Vijay, Omkar
</commit_message>
<xml_diff>
--- a/employees/employees.xlsx
+++ b/employees/employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Email Signature\employees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF9C713F-B206-404C-90CC-AA2B94D51563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D66419-FB9A-4E84-B562-F5905388B6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{13FF4E98-4AD7-478F-BA3A-EC3DF8F57A6B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>Name</t>
   </si>
@@ -132,6 +132,30 @@
   </si>
   <si>
     <t>Ramesh Ginde</t>
+  </si>
+  <si>
+    <t>anjan@abhinavinfra.com</t>
+  </si>
+  <si>
+    <t>Anjan Rout</t>
+  </si>
+  <si>
+    <t>hemant@abhinavinfra.com</t>
+  </si>
+  <si>
+    <t>Vijay Kakade</t>
+  </si>
+  <si>
+    <t>accounts@abhinavinfra.com</t>
+  </si>
+  <si>
+    <t>Hemant Adholkar</t>
+  </si>
+  <si>
+    <t>Omkar Mule</t>
+  </si>
+  <si>
+    <t>omkar@abhinavinfra.com</t>
   </si>
 </sst>
 </file>
@@ -531,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB07BDA-D330-4957-92CA-55A517FF57E1}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -680,6 +704,62 @@
         <v>30</v>
       </c>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>9970200123</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12">
+        <v>9225536268</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13">
+        <v>9881479770</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14">
+        <v>9881062695</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="mailto:ai@abhinavinfra.com" xr:uid="{A2A4E5CA-6F11-46F4-9BC1-43D51792CDF8}"/>
@@ -691,6 +771,10 @@
     <hyperlink ref="D8" r:id="rId7" xr:uid="{06DAB31C-2358-4C74-8222-424634A312A0}"/>
     <hyperlink ref="D9" r:id="rId8" xr:uid="{F48D1BA6-49DC-45CA-98BA-E5EAE552BEA2}"/>
     <hyperlink ref="D10" r:id="rId9" xr:uid="{5AE1A901-293E-4DA2-A073-C642276F0C34}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{A1545729-2313-4E26-AAD0-C98055998132}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{6A7CFDC3-FA9B-4E88-B46D-5BA0AE94D9F2}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{BB927F65-71DB-4DE5-8C2B-77203F31AAEA}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{B049B222-6DE9-4550-9369-E20A7C6B230E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add email signature for SHANKAR S. AAMBURE
</commit_message>
<xml_diff>
--- a/employees/employees.xlsx
+++ b/employees/employees.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -766,6 +766,26 @@
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>omkar@abhinavinfra.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SHANKAR S. AAMBURE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Manager- Planning &amp; Project Coordination</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7219552280</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>planning@abhinavinfra.com</t>
         </is>
       </c>
     </row>

</xml_diff>